<commit_message>
Reporte Integrado BORA-COMPRAR-TGN: 2026-03-12
</commit_message>
<xml_diff>
--- a/data/2026-03/flujo_licitaciones_2026-03-12.xlsx
+++ b/data/2026-03/flujo_licitaciones_2026-03-12.xlsx
@@ -656,22 +656,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>40/5-0102-CDI26</t>
+          <t>84/30-0126-LPR26</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MANTENIMIENTO, REPARACION, LIMPIEZA, RECARGA Y PRUEBA HIDRAULICA DE MATAFUEGOS</t>
+          <t>Contratacion del Servicio de Protocolo y Ceremonial</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>12/03/2026 08:00 Hrs.</t>
+          <t>12/03/2026 09:00 Hrs.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>40/005 - BASE AEREA MILITAR MORON</t>
+          <t>84/30 - Liceo Militar General Paz</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -703,22 +703,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>40/16-0027-LPR26</t>
+          <t>40/19-0135-CDI26</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE VERDURAS PARA LA ELABORACIÓN DE ALIMENTOS</t>
+          <t>ADQUISICION INSUMOS E INSTRUMENTAL ODONTOLOGICO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Contratación Directa</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>12/03/2026 08:00 Hrs.</t>
+          <t>12/03/2026 09:00 Hrs.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>40/016 - AREA MATERIAL QUILMES</t>
+          <t>40/019 - UOC  RTA</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -750,17 +750,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>84/30-0126-LPR26</t>
+          <t>37/19-0051-CDI26</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Contratacion del Servicio de Protocolo y Ceremonial</t>
+          <t>ADQUISICIÓN DE INSUMOS MÉDICOS Y ODONTOLÓGICOS</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Contratación Directa</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>84/30 - Liceo Militar General Paz</t>
+          <t>37/019 - Jefatura De Agrupación V "Entre Rios"</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>40/19-0135-CDI26</t>
+          <t>74/29-0045-LPR26</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ADQUISICION INSUMOS E INSTRUMENTAL ODONTOLOGICO</t>
+          <t>Adquisicion de caja de direccion para móvil oficial del Parque Nacional Laguna Blanca</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>40/019 - UOC  RTA</t>
+          <t>74/29 - Parque Nacional Laguna Blanca</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -844,12 +844,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>37/19-0051-CDI26</t>
+          <t>47-0014-CDI26</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE INSUMOS MÉDICOS Y ODONTOLÓGICOS</t>
+          <t>Servicio de mano de obra con provisión de materiales cambio de piso en terraza del Edificio INIDEP</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>12/03/2026 09:00 Hrs.</t>
+          <t>12/03/2026 10:00 Hrs.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>37/019 - Jefatura De Agrupación V "Entre Rios"</t>
+          <t>47 - Dpto. de Compras y Servicios- INIDEP</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -891,22 +891,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>74/29-0045-LPR26</t>
+          <t>37/134-0305-CDI26</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Adquisicion de caja de direccion para móvil oficial del Parque Nacional Laguna Blanca</t>
+          <t>ADQUISICION DEL SERVICIO DE DOSIMETRÍA Y RESIDUOS PATÓGENOS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Contratación Directa</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>12/03/2026 09:00 Hrs.</t>
+          <t>12/03/2026 10:00 Hrs.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>74/29 - Parque Nacional Laguna Blanca</t>
+          <t>37/134 - SERVICIO ADMINISTRATIVO FINANCIERO DESCONCENTRADO "ESCUADRÓN 65 CORDOBA"</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -938,12 +938,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>47-0014-CDI26</t>
+          <t>37/67-1089-CDI25</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Servicio de mano de obra con provisión de materiales cambio de piso en terraza del Edificio INIDEP</t>
+          <t>ADQUISICIÓN DE TÓNER</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>47 - Dpto. de Compras y Servicios- INIDEP</t>
+          <t>37/067 - Escuadrón 39 "Perito Moreno"</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -985,12 +985,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>37/134-0305-CDI26</t>
+          <t>37/17-0192-CDI26</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ADQUISICION DEL SERVICIO DE DOSIMETRÍA Y RESIDUOS PATÓGENOS</t>
+          <t>ADQUISICIÓN DE SERVICIO PARA MANTENIMIENTO Y RECARGA DE MATAFUEGOS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>37/134 - SERVICIO ADMINISTRATIVO FINANCIERO DESCONCENTRADO "ESCUADRÓN 65 CORDOBA"</t>
+          <t>37/017 - Escuadrón 47 "Ituzaingo"</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1032,12 +1032,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>37/67-1089-CDI25</t>
+          <t>37/68-1232-CDI25</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE TÓNER</t>
+          <t>ADQUISICIÓN DE INSUMOS VETERINARIOS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>37/067 - Escuadrón 39 "Perito Moreno"</t>
+          <t>37/068 - Escuadrón 42 "Calafate"</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>37/17-0192-CDI26</t>
+          <t>37/33-0119-CDI26</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE SERVICIO PARA MANTENIMIENTO Y RECARGA DE MATAFUEGOS</t>
+          <t>ADQUISICIÓN DE ELEMENTOS DE LIMPIEZA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>37/017 - Escuadrón 47 "Ituzaingo"</t>
+          <t>37/033 - Escuadron 18 "Lomitas"</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">

</xml_diff>